<commit_message>
Separate D3 D4 reference qualification from cross-dimension scores
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D3 Physical rationality and rate constraints/outputs/data/D3_sensor_summary.xlsx
+++ b/Project 1 Data Quality Assessment/D3 Physical rationality and rate constraints/outputs/data/D3_sensor_summary.xlsx
@@ -181,7 +181,7 @@
     <t>soft_bound</t>
   </si>
   <si>
-    <t>v2.7.0</t>
+    <t>v2.8.0</t>
   </si>
 </sst>
 </file>
@@ -672,37 +672,37 @@
         <v>0.9959147135416667</v>
       </c>
       <c r="G2">
-        <v>4.964634239289305</v>
+        <v>4.975188110774293</v>
       </c>
       <c r="H2">
         <v>5</v>
       </c>
       <c r="I2">
-        <v>3.179518045560728</v>
+        <v>3.182345351480197</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>0.02667105696410932</v>
+        <v>0.01481725386894962</v>
       </c>
       <c r="L2">
-        <v>0.05202502469542312</v>
+        <v>0.06025683240039513</v>
       </c>
       <c r="M2">
         <v>0.004231770833333333</v>
       </c>
       <c r="N2">
-        <v>0.02766927083333333</v>
+        <v>0.01432291666666667</v>
       </c>
       <c r="O2">
         <v>9.156512909776618E-05</v>
       </c>
       <c r="P2">
-        <v>0.008297976501305485</v>
+        <v>0.003815818102697998</v>
       </c>
       <c r="Q2">
-        <v>0.008360736599802698</v>
+        <v>0.00384467828565165</v>
       </c>
       <c r="R2">
         <v>0.991742819843342</v>
@@ -750,7 +750,7 @@
         <v>0</v>
       </c>
       <c r="AG2">
-        <v>0.07869608165953243</v>
+        <v>0.07507408626934475</v>
       </c>
       <c r="AH2">
         <v>0.0003292723081988805</v>
@@ -782,37 +782,37 @@
         <v>0.9959201388888889</v>
       </c>
       <c r="G3">
-        <v>4.93178496289583</v>
+        <v>4.95739729486909</v>
       </c>
       <c r="H3">
         <v>5</v>
       </c>
       <c r="I3">
-        <v>3.161787143765561</v>
+        <v>3.340564444794301</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>0.0642081000987817</v>
+        <v>0.01712216002634178</v>
       </c>
       <c r="L3">
-        <v>0.1402700032927231</v>
+        <v>0.1639776094830425</v>
       </c>
       <c r="M3">
         <v>0</v>
       </c>
       <c r="N3">
-        <v>0.06673177083333333</v>
+        <v>0.01985677083333333</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>0.01285628807658834</v>
+        <v>0.004422323759791123</v>
       </c>
       <c r="Q3">
-        <v>0.01295352406006796</v>
+        <v>0.004455771127918448</v>
       </c>
       <c r="R3">
         <v>0.991742819843342</v>
@@ -860,7 +860,7 @@
         <v>0</v>
       </c>
       <c r="AG3">
-        <v>0.2044781033915048</v>
+        <v>0.1810997695093843</v>
       </c>
       <c r="AH3">
         <v>0.0009878169245966415</v>
@@ -913,16 +913,16 @@
         <v>0</v>
       </c>
       <c r="N4">
-        <v>0.0029296875</v>
+        <v>0.0003255208333333333</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>0.0007968885987815492</v>
+        <v>1.087902523933855E-05</v>
       </c>
       <c r="Q4">
-        <v>0.0008029157075523404</v>
+        <v>1.096130658774526E-05</v>
       </c>
       <c r="R4">
         <v>0.991742819843342</v>
@@ -1109,37 +1109,37 @@
         <v>0.9959092881944445</v>
       </c>
       <c r="G6">
-        <v>4.93648979343922</v>
+        <v>4.963148323147151</v>
       </c>
       <c r="H6">
         <v>5</v>
       </c>
       <c r="I6">
-        <v>3.241887004861091</v>
+        <v>3.241892586006434</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>0.05070793546262759</v>
+        <v>0.02634178465591044</v>
       </c>
       <c r="L6">
-        <v>0.0388541323674679</v>
+        <v>0.04346394468225222</v>
       </c>
       <c r="M6">
         <v>0</v>
       </c>
       <c r="N6">
-        <v>0.05110677083333334</v>
+        <v>0.02604166666666667</v>
       </c>
       <c r="O6">
         <v>0</v>
       </c>
       <c r="P6">
-        <v>0.02062729465154208</v>
+        <v>0.0107327297759835</v>
       </c>
       <c r="Q6">
-        <v>0.02078330510106048</v>
+        <v>0.01081390464768611</v>
       </c>
       <c r="R6">
         <v>0.991742819843342</v>
@@ -1187,7 +1187,7 @@
         <v>0</v>
       </c>
       <c r="AG6">
-        <v>0.08956206783009549</v>
+        <v>0.06980572933816266</v>
       </c>
       <c r="AH6">
         <v>0.001317089232795522</v>
@@ -1219,37 +1219,37 @@
         <v>0.9959038628472223</v>
       </c>
       <c r="G7">
-        <v>4.956801614236591</v>
+        <v>4.974403147919013</v>
       </c>
       <c r="H7">
         <v>5</v>
       </c>
       <c r="I7">
-        <v>3.359895220673947</v>
+        <v>3.360005393459578</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>0.0388541323674679</v>
+        <v>0.01843924925913731</v>
       </c>
       <c r="L7">
-        <v>0.0135001646361541</v>
+        <v>0.01448798156075074</v>
       </c>
       <c r="M7">
         <v>0</v>
       </c>
       <c r="N7">
-        <v>0.03841145833333334</v>
+        <v>0.01822916666666667</v>
       </c>
       <c r="O7">
         <v>0</v>
       </c>
       <c r="P7">
-        <v>0.01709993070335184</v>
+        <v>0.00991682573812815</v>
       </c>
       <c r="Q7">
-        <v>0.0172292626356692</v>
+        <v>0.009991829681560227</v>
       </c>
       <c r="R7">
         <v>0.991742819843342</v>
@@ -1297,7 +1297,7 @@
         <v>0</v>
       </c>
       <c r="AG7">
-        <v>0.05235429700362199</v>
+        <v>0.03292723081988805</v>
       </c>
       <c r="AH7">
         <v>0.0009878169245966415</v>
@@ -1350,16 +1350,16 @@
         <v>0</v>
       </c>
       <c r="N8">
-        <v>0.4508463541666667</v>
+        <v>0.0068359375</v>
       </c>
       <c r="O8">
         <v>0</v>
       </c>
       <c r="P8">
-        <v>0.05474846459088568</v>
+        <v>0.0009437554395126197</v>
       </c>
       <c r="Q8">
-        <v>0.0551625437377421</v>
+        <v>0.0009508933464869012</v>
       </c>
       <c r="R8">
         <v>0.991742796988247</v>

</xml_diff>